<commit_message>
Adiciona vitrine afiliada e criativos da fase 2
</commit_message>
<xml_diff>
--- a/docs/MobilyTech_Fase2_Finalistas_Validacao_Criativos_2026-06-13.xlsx
+++ b/docs/MobilyTech_Fase2_Finalistas_Validacao_Criativos_2026-06-13.xlsx
@@ -1434,14 +1434,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="51" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="57" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1487,12 +1487,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/case-ssd-nvme-01.svg</t>
+          <t>./assets/phase2-creatives/case-ssd-nvme-01.jpg</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
@@ -1512,37 +1512,37 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/case-ssd-nvme-02.svg</t>
+          <t>./assets/phase2-creatives/case-ssd-nvme-02.jpg</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Case SSD/HD SATA 2.5 USB 3.0</t>
+          <t>Case SSD M.2 NVMe USB-C 10Gbps</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nao jogue fora o HD antigo: transforme em backup externo</t>
+          <t>Oferta e chamada para Mercado Livre</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/case-ssd-sata-01.svg</t>
+          <t>./assets/phase2-creatives/case-ssd-nvme-03.jpg</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>selecionado para vitrine</t>
         </is>
       </c>
     </row>
@@ -1553,78 +1553,78 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Upgrade simples para quem comprou PC revisado</t>
+          <t>Nao jogue fora o HD antigo: transforme em backup externo</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/case-ssd-sata-02.svg</t>
+          <t>./assets/phase2-creatives/case-ssd-sata-01.jpg</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Fone KZ Castor monitor in-ear</t>
+          <t>Case SSD/HD SATA 2.5 USB 3.0</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Som de monitor gastando menos que headset gamer comum</t>
+          <t>Upgrade simples para quem comprou PC revisado</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/fone-kz-castor-01.svg</t>
+          <t>./assets/phase2-creatives/case-ssd-sata-02.jpg</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Fone KZ Castor monitor in-ear</t>
+          <t>Case SSD/HD SATA 2.5 USB 3.0</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Setup limpo para jogar, estudar e ouvir musica</t>
+          <t>Oferta e chamada para Mercado Livre</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/fone-kz-castor-02.svg</t>
+          <t>./assets/phase2-creatives/case-ssd-sata-03.jpg</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>selecionado para vitrine</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Kit limpeza ESD antiestatico para PC</t>
+          <t>Fone KZ Castor monitor in-ear</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -1632,24 +1632,24 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Poeira e estatica: o erro silencioso que mata desempenho</t>
+          <t>Som de monitor gastando menos que headset gamer comum</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/kit-limpeza-esd-01.svg</t>
+          <t>./assets/phase2-creatives/fone-kz-castor-01.jpg</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kit limpeza ESD antiestatico para PC</t>
+          <t>Fone KZ Castor monitor in-ear</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1657,124 +1657,124 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Kit simples para manter teclado, placa e gabinete apresentaveis</t>
+          <t>Setup limpo para jogar, estudar e ouvir musica</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/kit-limpeza-esd-02.svg</t>
+          <t>./assets/phase2-creatives/fone-kz-castor-02.jpg</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mini aspirador USB para teclado e cantos do setup</t>
+          <t>Fone KZ Castor monitor in-ear</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Teclado cheio de migalha e poeira em 30 segundos</t>
+          <t>Oferta e chamada para Mercado Livre</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/mini-aspirador-teclado-01.svg</t>
+          <t>./assets/phase2-creatives/fone-kz-castor-03.jpg</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>selecionado para vitrine</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mini aspirador USB para teclado e cantos do setup</t>
+          <t>Kit limpeza ESD antiestatico para PC</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Limpeza rapida para mesa, notebook e setup gamer</t>
+          <t>Poeira e estatica: o erro silencioso que mata desempenho</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/mini-aspirador-teclado-02.svg</t>
+          <t>./assets/phase2-creatives/kit-limpeza-esd-01.jpg</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Hub USB-C 4 portas para notebook e celular</t>
+          <t>Kit limpeza ESD antiestatico para PC</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Falta porta USB no notebook? Resolva sem gambiarra</t>
+          <t>Kit simples para manter teclado, placa e gabinete apresentaveis</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/hub-usb-c-01.svg</t>
+          <t>./assets/phase2-creatives/kit-limpeza-esd-02.jpg</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Hub USB-C 4 portas para notebook e celular</t>
+          <t>Kit limpeza ESD antiestatico para PC</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Mouse, teclado, pendrive e headset no mesmo hub</t>
+          <t>Oferta e chamada para Mercado Livre</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/hub-usb-c-02.svg</t>
+          <t>./assets/phase2-creatives/kit-limpeza-esd-03.jpg</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>selecionado para vitrine</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Suporte anti-sag para placa de video</t>
+          <t>Mini aspirador USB para teclado e cantos do setup</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1782,24 +1782,24 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Sua placa de video esta torta? Evite peso no slot PCIe</t>
+          <t>Teclado cheio de migalha e poeira em 30 segundos</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/suporte-gpu-antisag-01.svg</t>
+          <t>./assets/phase2-creatives/mini-aspirador-teclado-01.jpg</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Suporte anti-sag para placa de video</t>
+          <t>Mini aspirador USB para teclado e cantos do setup</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -1807,124 +1807,124 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Setup gamer mais limpo com suporte ajustavel</t>
+          <t>Limpeza rapida para mesa, notebook e setup gamer</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/suporte-gpu-antisag-02.svg</t>
+          <t>./assets/phase2-creatives/mini-aspirador-teclado-02.jpg</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>selecionado para vitrine</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kit keycaps PBT para teclado mecanico</t>
+          <t>Mini aspirador USB para teclado e cantos do setup</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Teclado antigo, cara nova em minutos</t>
+          <t>Oferta e chamada para Mercado Livre</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/keycaps-pbt-01.svg</t>
+          <t>./assets/phase2-creatives/mini-aspirador-teclado-03.jpg</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kit keycaps PBT para teclado mecanico</t>
+          <t>Hub USB-C 4 portas para notebook e celular</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Personalize o setup sem comprar teclado novo</t>
+          <t>Falta porta USB no notebook? Resolva sem gambiarra</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/keycaps-pbt-02.svg</t>
+          <t>./assets/phase2-creatives/hub-usb-c-01.jpg</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Teclado gamer mecanico RGB ABNT2</t>
+          <t>Hub USB-C 4 portas para notebook e celular</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Switch red, RGB e ABNT2 para jogar sem adaptacao</t>
+          <t>Mouse, teclado, pendrive e headset no mesmo hub</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/teclado-mecanico-abnt2-01.svg</t>
+          <t>./assets/phase2-creatives/hub-usb-c-02.jpg</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Teclado gamer mecanico RGB ABNT2</t>
+          <t>Hub USB-C 4 portas para notebook e celular</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>O upgrade mais visivel do setup</t>
+          <t>Oferta e chamada para Mercado Livre</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/teclado-mecanico-abnt2-02.svg</t>
+          <t>./assets/phase2-creatives/hub-usb-c-03.jpg</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>selecionado para vitrine</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Fita LED bias lighting USB para monitor</t>
+          <t>Suporte anti-sag para placa de video</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1932,24 +1932,24 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Deixe o monitor mais confortavel a noite</t>
+          <t>Sua placa de video esta torta? Evite peso no slot PCIe</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>./assets/phase2-creatives/bias-light-led-01.svg</t>
+          <t>./assets/phase2-creatives/suporte-gpu-antisag-01.jpg</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>rascunho para aprovacao</t>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Fita LED bias lighting USB para monitor</t>
+          <t>Suporte anti-sag para placa de video</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -1957,17 +1957,267 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
+          <t>Setup gamer mais limpo com suporte ajustavel</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/suporte-gpu-antisag-02.jpg</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Suporte anti-sag para placa de video</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Oferta e chamada para Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/suporte-gpu-antisag-03.jpg</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>selecionado para vitrine</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Kit keycaps PBT para teclado mecanico</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Teclado antigo, cara nova em minutos</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/keycaps-pbt-01.jpg</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Kit keycaps PBT para teclado mecanico</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Personalize o setup sem comprar teclado novo</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/keycaps-pbt-02.jpg</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Kit keycaps PBT para teclado mecanico</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Oferta e chamada para Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/keycaps-pbt-03.jpg</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>selecionado para vitrine</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Teclado gamer mecanico RGB ABNT2</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Switch red, RGB e ABNT2 para jogar sem adaptacao</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/teclado-mecanico-abnt2-01.jpg</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Teclado gamer mecanico RGB ABNT2</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>O upgrade mais visivel do setup</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/teclado-mecanico-abnt2-02.jpg</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Teclado gamer mecanico RGB ABNT2</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Oferta e chamada para Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/teclado-mecanico-abnt2-03.jpg</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>selecionado para vitrine</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Fita LED bias lighting USB para monitor</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Deixe o monitor mais confortavel a noite</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/bias-light-led-01.jpg</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Fita LED bias lighting USB para monitor</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>Setup com cara gamer gastando pouco</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>./assets/phase2-creatives/bias-light-led-02.svg</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>rascunho para aprovacao</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/bias-light-led-02.jpg</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>selecionado para vitrine</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Fita LED bias lighting USB para monitor</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Oferta e chamada para Mercado Livre</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>./assets/phase2-creatives/bias-light-led-03.jpg</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>alternativa para aprovacao</t>
         </is>
       </c>
     </row>
@@ -1997,7 +2247,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>2026-06-13 09:57:06</t>
+          <t>2026-06-13 12:07:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finaliza fase 2 MobilyTech e fluxo hibrido
</commit_message>
<xml_diff>
--- a/docs/MobilyTech_Fase2_Finalistas_Validacao_Criativos_2026-06-13.xlsx
+++ b/docs/MobilyTech_Fase2_Finalistas_Validacao_Criativos_2026-06-13.xlsx
@@ -601,7 +601,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Margem bruta alvo de R$40 a R$65 antes de trafego e taxas</t>
+          <t>Margem bruta alvo de R$40 a R$65 antes de taxas</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Margem bruta alvo de R$20 a R$35 antes de trafego e taxas</t>
+          <t>Margem bruta alvo de R$20 a R$35 antes de taxas</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Boa margem em kit/combo; trafego frio precisa criativo forte</t>
+          <t>Boa margem em kit/combo; campanha fria precisa criativo forte</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="57" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>alternativa para aprovacao</t>
+          <t>alternativa de criativo</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>2026-06-13 12:07:32</t>
+          <t>2026-06-13 23:59:30</t>
         </is>
       </c>
     </row>

</xml_diff>